<commit_message>
CORE-000008 edits made based on discussion board feedback.  Tests are passing.
</commit_message>
<xml_diff>
--- a/rules/CORE-000008/negative/01/data/unit-test-coreid-CG0132-negative.xlsx
+++ b/rules/CORE-000008/negative/01/data/unit-test-coreid-CG0132-negative.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -63,18 +63,9 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -88,18 +79,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -129,7 +108,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -137,8 +116,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,7 +509,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -571,32 +548,72 @@
         <v>DTHFL</v>
       </c>
       <c r="F2" s="4" t="str">
-        <v>[ABSENT]</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="4" t="str">
-        <v>dm.xpt</v>
+        <v>ss.xpt</v>
       </c>
       <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
       <c r="D3" s="4">
+        <v>5</v>
+      </c>
+      <c r="E3" s="4" t="str">
+        <v>SSSTRESC</v>
+      </c>
+      <c r="F3" s="4" t="str">
+        <v>DEAD</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C4" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="4">
         <v>6</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E4" s="4" t="str">
         <v>DTHFL</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F4" s="4" t="str">
         <v>N</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>ss.xpt</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="4">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <v>SSSTRESC</v>
+      </c>
+      <c r="F5" s="4" t="str">
+        <v>DEAD</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -692,248 +709,248 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="5" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="6" t="str">
+      <c r="M2" s="5" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="N2" s="5" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="6" t="str">
+      <c r="O2" s="5" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="6" t="str">
+      <c r="P2" s="5" t="str">
         <v>Age Text</v>
       </c>
-      <c r="Q2" s="6" t="str">
+      <c r="Q2" s="5" t="str">
         <v>Age Units</v>
       </c>
-      <c r="R2" s="6" t="str">
+      <c r="R2" s="5" t="str">
         <v>Sex</v>
       </c>
-      <c r="S2" s="6" t="str">
+      <c r="S2" s="5" t="str">
         <v>Race</v>
       </c>
-      <c r="T2" s="6" t="str">
+      <c r="T2" s="5" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="U2" s="6" t="str">
+      <c r="U2" s="5" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="V2" s="6" t="str">
+      <c r="V2" s="5" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="W2" s="6" t="str">
+      <c r="W2" s="5" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="X2" s="6" t="str">
+      <c r="X2" s="5" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="Y2" s="6" t="str">
+      <c r="Y2" s="5" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="Z2" s="6" t="str">
+      <c r="Z2" s="5" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="AA2" s="6" t="str">
+      <c r="AA2" s="5" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AA3" s="6" t="str">
+      <c r="P3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AA3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>20</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>12</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>10</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>10</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <v>10</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>10</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>10</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>10</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>10</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5">
         <v>1</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="5">
         <v>3</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="5">
         <v>10</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="5">
         <v>8</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="5">
         <v>5</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4" s="5">
         <v>5</v>
       </c>
-      <c r="R4" s="6">
+      <c r="R4" s="5">
         <v>1</v>
       </c>
-      <c r="S4" s="6">
+      <c r="S4" s="5">
         <v>41</v>
       </c>
-      <c r="T4" s="6">
+      <c r="T4" s="5">
         <v>22</v>
       </c>
-      <c r="U4" s="6">
+      <c r="U4" s="5">
         <v>8</v>
       </c>
-      <c r="V4" s="6">
+      <c r="V4" s="5">
         <v>28</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4" s="5">
         <v>8</v>
       </c>
-      <c r="X4" s="6">
+      <c r="X4" s="5">
         <v>28</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="5">
         <v>14</v>
       </c>
-      <c r="Z4" s="6">
+      <c r="Z4" s="5">
         <v>200</v>
       </c>
-      <c r="AA4" s="6">
+      <c r="AA4" s="5">
         <v>3</v>
       </c>
     </row>
@@ -971,7 +988,7 @@
       <c r="K5" s="4" t="str">
         <v>2021-02-18</v>
       </c>
-      <c r="L5" s="7" t="str">
+      <c r="L5" s="6" t="str">
         <v/>
       </c>
       <c r="M5" s="4" t="str">
@@ -1054,7 +1071,7 @@
       <c r="K6" s="4" t="str">
         <v>2018-09-04</v>
       </c>
-      <c r="L6" s="8" t="str">
+      <c r="L6" s="6" t="str">
         <v>N</v>
       </c>
       <c r="M6" s="4" t="str">
@@ -1233,111 +1250,111 @@
       </c>
     </row>
     <row r="2" xml:space="preserve">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Status Short Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Status Name</v>
       </c>
-      <c r="G2" s="6" t="str" xml:space="preserve">
+      <c r="G2" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">Result or Finding
 Original Result</v>
       </c>
-      <c r="H2" s="6" t="str" xml:space="preserve">
+      <c r="H2" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">Character
 Result/Finding in
 Std Format</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Epoch</v>
       </c>
-      <c r="K2" s="6" t="str" xml:space="preserve">
+      <c r="K2" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">Date/Time of
 Assessment</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>20</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>8</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>50</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <v>50</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>50</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>8</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>50</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>19</v>
       </c>
     </row>
@@ -1363,7 +1380,7 @@
       <c r="G5" s="4" t="str">
         <v>DEAD</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="6" t="str">
         <v>DEAD</v>
       </c>
       <c r="I5" s="4">
@@ -1398,7 +1415,7 @@
       <c r="G6" s="4" t="str">
         <v>DEAD</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="6" t="str">
         <v>DEAD</v>
       </c>
       <c r="I6" s="4">

</xml_diff>